<commit_message>
Add 12 source-reviewed Nankai profiles with explicit retirement, guidance types and visible teaching levels
</commit_message>
<xml_diff>
--- a/site/exports/nku-economics.xlsx
+++ b/site/exports/nku-economics.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导师'!$A$1:$L$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导师'!$A$1:$L$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -451,8 +451,8 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="65" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="30.8" customWidth="1" min="6" max="6"/>
-    <col width="37.8" customWidth="1" min="7" max="7"/>
+    <col width="65" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
     <col width="26.6" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
@@ -675,12 +675,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>关永强</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>校区未标注</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>经济学院</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>https://economics.nankai.edu.cn/2019/1006/c16878a208250/page.htm</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>当前人事与退休状态未独立核实；目录/至今/现任不作实时认证，导航和当前教师计数关闭。；必要职业摘录非完整网页、HTTP或论文原件；观察依据和精度按原记录，未外核书目出版元数据或全文。；学历获授、学习区间和授位日期分别保留；本人博导/硕导资格不用于生成本人的导师。；本科及硕博研究生仅学习标签，授位unknown；硕博2003-09至2009-06共一事件，不拆造两段日期或两获授。；张东刚仅共享硕博阶段导师；Kenneth Pomeranz及Johanna Bockman分别对应两访学合作导师，不升级学位论文关系。；2007联合培养/2019富布赖特VRS两访学为非学位事件，不声称访问院校授位；项目名按源保留。；经济学院为既有机构，复用原节点；经济研究所仅原归属标签保留，不推其法定行政父级或另造同义学院。</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；部分已留存职业资料，非完整履历或现职认证；公开教学事实（非本人求学学历；教学／课程开设时间不是入学、授位或任职起点；不计入教育、任职、论文、导师统计及师承图）：中国经济史；角色未披露；教学／课程开设时间：时间未披露；来源所列讲授课程，不保证观察日实际开授或独立主讲。按来源分组、层级及合上标签保留；不认证当前开课或单独主讲。 来源教学层级：本科。；来源ID：nku219-guan-profile；https://economics.nankai.edu.cn/2019/1006/c16878a208250/page.htm；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>公开个人页（访问与内容时效见来源记录）</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K4"/>
+  <autoFilter ref="A1:K5"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -692,13 +746,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:S21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="29.4" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="19.6" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
@@ -709,7 +763,7 @@
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="65" customWidth="1" min="14" max="14"/>
-    <col width="37.8" customWidth="1" min="15" max="15"/>
+    <col width="65" customWidth="1" min="15" max="15"/>
     <col width="28" customWidth="1" min="16" max="16"/>
     <col width="65" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
@@ -1968,8 +2022,337 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>关永强</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>degree_study</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>1996-09</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>2000-06</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>世界经济</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>仅本科/研究生学习阶段，无明确获授；硕博共享2003.9-2009.6区间，不拆造两段起止或学位日期。</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr"/>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>https://economics.nankai.edu.cn/2019/1006/c16878a208250/page.htm</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>关永强</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>degree_study</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>硕士、博士研究生（共享区间）</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2003-09</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>2009-06</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>经济史</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>仅本科/研究生学习阶段，无明确获授；硕博共享2003.9-2009.6区间，不拆造两段起止或学位日期。</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr"/>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>https://economics.nankai.edu.cn/2019/1006/c16878a208250/page.htm</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S18" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>关永强</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>visiting_research</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>访学（非学位）</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>美国加州大学尔湾分校（UCI）</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>2007-09</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>2008-09</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>访学/联合培养为该阶段非学位经历，不据此认定访问院校授位。</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr"/>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>https://economics.nankai.edu.cn/2019/1006/c16878a208250/page.htm</t>
+        </is>
+      </c>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S19" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>关永强</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>visiting_research</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>访学（非学位）</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>美国乔治梅森大学（GMU）</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>2019-08</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>2020-07</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>访学/联合培养为该阶段非学位经历，不据此认定访问院校授位。</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr"/>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>https://economics.nankai.edu.cn/2019/1006/c16878a208250/page.htm</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>关永强</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>教授</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>2021-12</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>开放终点原样保留，不自动解释为今天仍在职。</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>https://economics.nankai.edu.cn/2019/1006/c16878a208250/page.htm</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S16"/>
+  <autoFilter ref="A1:S21"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId2"/>
@@ -1987,6 +2370,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1998,18 +2386,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22.4" customWidth="1" min="2" max="2"/>
+    <col width="19.6" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="50.4" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="23.8" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="65" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
@@ -2077,8 +2465,163 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>关永强</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>张东刚</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>硕士、博士研究生（共享区间）</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>来源仅限硕士、博士研究生（共享区间）的指导关系；不升级正式学位论文导师。</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>导师身份节点及当前任职未独立确认。</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>https://economics.nankai.edu.cn/2019/1006/c16878a208250/page.htm</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>关永强</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Kenneth Pomeranz</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>UCI历史系访学/联合培养</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>来源仅限UCI历史系访学/联合培养的指导关系；不升级正式学位论文导师。</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>导师身份节点及当前任职未独立确认。</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>https://economics.nankai.edu.cn/2019/1006/c16878a208250/page.htm</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>关永强</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Johanna Bockman</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>GMU全球事务系访学</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>来源仅限GMU全球事务系访学的指导关系；不升级正式学位论文导师。</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>导师身份节点及当前任职未独立确认。</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>https://economics.nankai.edu.cn/2019/1006/c16878a208250/page.htm</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:L4"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId3"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2089,19 +2632,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="23.8" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
+    <col width="54.59999999999999" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="65" customWidth="1" min="9" max="9"/>
+    <col width="65" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
@@ -2168,8 +2711,118 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>关永强</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>近代中国的收入分配：一个定量的研究</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>https://economics.nankai.edu.cn/2019/1006/c16878a208250/page.htm</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>官网职业书目；monograph_as_official_list</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>https://economics.nankai.edu.cn/2019/1006/c16878a208250/page.htm</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>仅官网书目；未核出版元数据或全文。；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>作者、年份与作品类型只据该官网条目；不把转载年份替代原作年，不推额外角色。 来源贡献角色：listed_author；不由书目推师承。源出版地北京，时间2012年10月，不仅年份。</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>关永强</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>近代中国工资与生活费指数考略</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>https://economics.nankai.edu.cn/2019/1006/c16878a208250/page.htm</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>官网职业书目；journal_article_as_official_list</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>https://economics.nankai.edu.cn/2019/1006/c16878a208250/page.htm</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>仅官网书目；未核出版元数据或全文。；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>作者、年份与作品类型只据该官网条目；不把转载年份替代原作年，不推额外角色。 来源贡献角色：listed_author；不由书目推师承。</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:L3"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId4"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2180,13 +2833,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="39.2" customWidth="1" min="2" max="2"/>
     <col width="65" customWidth="1" min="3" max="3"/>
-    <col width="60.2" customWidth="1" min="4" max="4"/>
+    <col width="65" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
@@ -2454,27 +3107,27 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>包群</t>
+          <t>关永强</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>institution-classification-2</t>
+          <t>nku219-guan-profile</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</t>
+          <t>https://economics.nankai.edu.cn/2019/1006/c16878a208250/page.htm</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>历史985院校分类参考；非个人授位或就读当年建设身份的证明</t>
+          <t>既有必要职业摘录复核；非新抓取、完整网页或实时在岗认证；retained_professional_excerpts_checked</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>未单独记录</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -2491,42 +3144,116 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>关永强</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>nku219-guan-directory</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>https://economics.nankai.edu.cn/axs/list.htm</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>既有必要职业摘录复核；非新抓取、完整网页或实时在岗认证；retained_professional_excerpts_checked</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>包群</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>institution-classification-2</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>历史985院校分类参考；非个人授位或就读当年建设身份的证明</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>未单独记录</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>成前</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>institution-classification-2</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>历史985院校分类参考；非个人授位或就读当年建设身份的证明</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>未单独记录</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>nku</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>南开大学</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G9"/>
+  <autoFilter ref="A1:G11"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -2536,6 +3263,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>